<commit_message>
Add some more of the raw excel analysis
</commit_message>
<xml_diff>
--- a/2025/battwatts_sensitivity/battwatts_sensitivity_outputs_shade_todiscuss_v2.xlsx
+++ b/2025/battwatts_sensitivity/battwatts_sensitivity_outputs_shade_todiscuss_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bspeetle/Desktop/repo/SAM-analyses/2025/battwatts_sensitivity/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bmirletz\source\repos\sam_dev\SAM-analyses\2025\battwatts_sensitivity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{5E131F65-FE03-E447-AE3D-B5AC356AA28F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31CBE448-8CA3-41FB-8FF8-B590B7CE5B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20420" xr2:uid="{0BF71174-60D2-864F-9DF0-C456186B9F38}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0BF71174-60D2-864F-9DF0-C456186B9F38}"/>
   </bookViews>
   <sheets>
     <sheet name="battwatts_sensitivity_outputs_s" sheetId="1" r:id="rId1"/>
@@ -128,7 +128,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -608,11 +608,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="20" builtinId="30" customBuiltin="1"/>
@@ -989,26 +990,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B144A90-34B1-AC42-BC3E-0AD4CBB1EAC6}">
-  <dimension ref="A1:V37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Z37"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="8" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.1640625" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="22.1640625" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="30.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.125" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="22.125" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="30.375" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="29.5" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="26.33203125" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.375" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="26.375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="27" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="0" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="31.1640625" hidden="1" customWidth="1"/>
-    <col min="19" max="19" width="28.1640625" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="24.83203125" customWidth="1"/>
-    <col min="22" max="22" width="35.5" customWidth="1"/>
+    <col min="17" max="17" width="30.625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="31.125" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="28.125" hidden="1" customWidth="1"/>
+    <col min="21" max="22" width="24.875" customWidth="1"/>
+    <col min="23" max="23" width="35.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1069,11 +1070,11 @@
       <c r="U1" t="s">
         <v>27</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1135,12 +1136,21 @@
         <f>H2-N2</f>
         <v>-2.5749597479709792</v>
       </c>
-      <c r="V2" s="3">
+      <c r="V2" s="4">
+        <f>U2/H2</f>
+        <v>-2.9558442608080071E-3</v>
+      </c>
+      <c r="W2" s="3">
         <f>K2-Q2</f>
         <v>37.832083858199894</v>
       </c>
+      <c r="X2" s="4">
+        <f>W2/K2</f>
+        <v>3.4462820990703254E-2</v>
+      </c>
+      <c r="Y2" s="4"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -1202,12 +1212,21 @@
         <f t="shared" ref="U3:U37" si="0">H3-N3</f>
         <v>-1.7313991717610406</v>
       </c>
-      <c r="V3" s="3">
-        <f t="shared" ref="V3:V37" si="1">K3-Q3</f>
+      <c r="V3" s="4">
+        <f t="shared" ref="V3:V37" si="1">U3/H3</f>
+        <v>-1.9697394778703347E-3</v>
+      </c>
+      <c r="W3" s="3">
+        <f t="shared" ref="W3:W37" si="2">K3-Q3</f>
         <v>-54.48472166102988</v>
       </c>
+      <c r="X3" s="4">
+        <f t="shared" ref="X3:X37" si="3">W3/K3</f>
+        <v>-4.7071599206846212E-2</v>
+      </c>
+      <c r="Y3" s="4"/>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -1269,12 +1288,21 @@
         <f t="shared" si="0"/>
         <v>-2.0385665821210068</v>
       </c>
-      <c r="V4" s="3">
+      <c r="V4" s="4">
         <f t="shared" si="1"/>
+        <v>-2.3466455463879571E-3</v>
+      </c>
+      <c r="W4" s="3">
+        <f t="shared" si="2"/>
         <v>-16.42132087869004</v>
       </c>
+      <c r="X4" s="4">
+        <f t="shared" si="3"/>
+        <v>-1.4807891119482539E-2</v>
+      </c>
+      <c r="Y4" s="4"/>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1336,12 +1364,21 @@
         <f t="shared" si="0"/>
         <v>-2.8022103035290229</v>
       </c>
-      <c r="V5" s="3">
+      <c r="V5" s="4">
         <f t="shared" si="1"/>
+        <v>-3.1897141740396709E-3</v>
+      </c>
+      <c r="W5" s="3">
+        <f t="shared" si="2"/>
         <v>-32.611838426039867</v>
       </c>
+      <c r="X5" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.8281837334555499E-2</v>
+      </c>
+      <c r="Y5" s="4"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1403,12 +1440,25 @@
         <f t="shared" si="0"/>
         <v>-2.4305599383239951</v>
       </c>
-      <c r="V6" s="3">
+      <c r="V6" s="4">
         <f t="shared" si="1"/>
+        <v>-2.8654082152493169E-3</v>
+      </c>
+      <c r="W6" s="3">
+        <f t="shared" si="2"/>
         <v>-2.7893145401999391</v>
       </c>
+      <c r="X6" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.6849997498260255E-3</v>
+      </c>
+      <c r="Y6" s="4"/>
+      <c r="Z6" s="4">
+        <f>AVERAGE(X2:X13)</f>
+        <v>-2.1078187762570127E-2</v>
+      </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1470,12 +1520,21 @@
         <f t="shared" si="0"/>
         <v>-3.3377734168790312</v>
       </c>
-      <c r="V7" s="3">
+      <c r="V7" s="4">
         <f t="shared" si="1"/>
+        <v>-3.6848140344213991E-3</v>
+      </c>
+      <c r="W7" s="3">
+        <f t="shared" si="2"/>
         <v>-12.811454196890054</v>
       </c>
+      <c r="X7" s="4">
+        <f t="shared" si="3"/>
+        <v>-1.0710375695239095E-2</v>
+      </c>
+      <c r="Y7" s="4"/>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1537,12 +1596,21 @@
         <f t="shared" si="0"/>
         <v>-2.5276013246830189</v>
       </c>
-      <c r="V8" s="3">
+      <c r="V8" s="4">
         <f t="shared" si="1"/>
+        <v>-2.9594303160587047E-3</v>
+      </c>
+      <c r="W8" s="3">
+        <f t="shared" si="2"/>
         <v>-61.677394540520027</v>
       </c>
+      <c r="X8" s="4">
+        <f t="shared" si="3"/>
+        <v>-5.7230384685158973E-2</v>
+      </c>
+      <c r="Y8" s="4"/>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1604,12 +1672,21 @@
         <f t="shared" si="0"/>
         <v>-3.0898546198909571</v>
       </c>
-      <c r="V9" s="3">
+      <c r="V9" s="4">
         <f t="shared" si="1"/>
+        <v>-3.4972199857463953E-3</v>
+      </c>
+      <c r="W9" s="3">
+        <f t="shared" si="2"/>
         <v>-59.220396129810069</v>
       </c>
+      <c r="X9" s="4">
+        <f t="shared" si="3"/>
+        <v>-5.2461472344948634E-2</v>
+      </c>
+      <c r="Y9" s="4"/>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1671,12 +1748,21 @@
         <f t="shared" si="0"/>
         <v>-2.8044107382489756</v>
       </c>
-      <c r="V10" s="3">
+      <c r="V10" s="4">
         <f t="shared" si="1"/>
+        <v>-3.2749036117111717E-3</v>
+      </c>
+      <c r="W10" s="3">
+        <f t="shared" si="2"/>
         <v>-28.543511072939964</v>
       </c>
+      <c r="X10" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.6398929148557394E-2</v>
+      </c>
+      <c r="Y10" s="4"/>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1738,12 +1824,21 @@
         <f t="shared" si="0"/>
         <v>-2.7798749136040897</v>
       </c>
-      <c r="V11" s="3">
+      <c r="V11" s="4">
         <f t="shared" si="1"/>
+        <v>-3.1673012730508124E-3</v>
+      </c>
+      <c r="W11" s="3">
+        <f t="shared" si="2"/>
         <v>-57.762546082350127</v>
       </c>
+      <c r="X11" s="4">
+        <f t="shared" si="3"/>
+        <v>-4.8895579891953624E-2</v>
+      </c>
+      <c r="Y11" s="4"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1805,12 +1900,21 @@
         <f t="shared" si="0"/>
         <v>-2.2521954241310596</v>
       </c>
-      <c r="V12" s="3">
+      <c r="V12" s="4">
         <f t="shared" si="1"/>
+        <v>-2.6010338589470662E-3</v>
+      </c>
+      <c r="W12" s="3">
+        <f t="shared" si="2"/>
         <v>-2.194424124779971</v>
       </c>
+      <c r="X12" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.0418275925738298E-3</v>
+      </c>
+      <c r="Y12" s="4"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1872,12 +1976,21 @@
         <f t="shared" si="0"/>
         <v>-2.654638044936064</v>
       </c>
-      <c r="V13" s="3">
+      <c r="V13" s="4">
         <f t="shared" si="1"/>
+        <v>-2.9948779740345179E-3</v>
+      </c>
+      <c r="W13" s="3">
+        <f t="shared" si="2"/>
         <v>3.7890282220698737</v>
       </c>
+      <c r="X13" s="4">
+        <f t="shared" si="3"/>
+        <v>3.1838226275971086E-3</v>
+      </c>
+      <c r="Y13" s="4"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1939,12 +2052,25 @@
         <f t="shared" si="0"/>
         <v>-13.365091454989852</v>
       </c>
-      <c r="V14" s="3">
+      <c r="V14" s="4">
         <f t="shared" si="1"/>
+        <v>-5.9893644394286988E-3</v>
+      </c>
+      <c r="W14" s="3">
+        <f t="shared" si="2"/>
         <v>-55.561145705679792</v>
       </c>
+      <c r="X14" s="4">
+        <f t="shared" si="3"/>
+        <v>-1.6305612132342589E-2</v>
+      </c>
+      <c r="Y14" s="4"/>
+      <c r="Z14" s="4">
+        <f>AVERAGE(X14:X25)</f>
+        <v>-2.0411416672056013E-2</v>
+      </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -2006,12 +2132,21 @@
         <f t="shared" si="0"/>
         <v>-13.111593344149696</v>
       </c>
-      <c r="V15" s="3">
+      <c r="V15" s="4">
         <f t="shared" si="1"/>
+        <v>-5.812152741587826E-3</v>
+      </c>
+      <c r="W15" s="3">
+        <f t="shared" si="2"/>
         <v>-66.339019368910158</v>
       </c>
+      <c r="X15" s="4">
+        <f t="shared" si="3"/>
+        <v>-1.9119053032388107E-2</v>
+      </c>
+      <c r="Y15" s="4"/>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -2073,12 +2208,21 @@
         <f t="shared" si="0"/>
         <v>-10.107960938630185</v>
       </c>
-      <c r="V16" s="3">
+      <c r="V16" s="4">
         <f t="shared" si="1"/>
+        <v>-4.6277432716852742E-3</v>
+      </c>
+      <c r="W16" s="3">
+        <f t="shared" si="2"/>
         <v>-64.332304765069694</v>
       </c>
+      <c r="X16" s="4">
+        <f t="shared" si="3"/>
+        <v>-1.9167721077418425E-2</v>
+      </c>
+      <c r="Y16" s="4"/>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -2140,12 +2284,21 @@
         <f t="shared" si="0"/>
         <v>-12.711305194090073</v>
       </c>
-      <c r="V17" s="3">
+      <c r="V17" s="4">
         <f t="shared" si="1"/>
+        <v>-5.6575952614798183E-3</v>
+      </c>
+      <c r="W17" s="3">
+        <f t="shared" si="2"/>
         <v>-47.108838713779733</v>
       </c>
+      <c r="X17" s="4">
+        <f t="shared" si="3"/>
+        <v>-1.3577283243856479E-2</v>
+      </c>
+      <c r="Y17" s="4"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -2207,12 +2360,21 @@
         <f t="shared" si="0"/>
         <v>-15.276410152360313</v>
       </c>
-      <c r="V18" s="3">
+      <c r="V18" s="4">
         <f t="shared" si="1"/>
+        <v>-6.581990299073746E-3</v>
+      </c>
+      <c r="W18" s="3">
+        <f t="shared" si="2"/>
         <v>-74.450654005469914</v>
       </c>
+      <c r="X18" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.1395739251642225E-2</v>
+      </c>
+      <c r="Y18" s="4"/>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -2274,12 +2436,21 @@
         <f t="shared" si="0"/>
         <v>-17.61500298116016</v>
       </c>
-      <c r="V19" s="3">
+      <c r="V19" s="4">
         <f t="shared" si="1"/>
+        <v>-7.2687367522076317E-3</v>
+      </c>
+      <c r="W19" s="3">
+        <f t="shared" si="2"/>
         <v>-77.839599633950002</v>
       </c>
+      <c r="X19" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.1464219819290628E-2</v>
+      </c>
+      <c r="Y19" s="4"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -2341,12 +2512,21 @@
         <f t="shared" si="0"/>
         <v>-13.598895337069735</v>
       </c>
-      <c r="V20" s="3">
+      <c r="V20" s="4">
         <f t="shared" si="1"/>
+        <v>-6.0515098740649914E-3</v>
+      </c>
+      <c r="W20" s="3">
+        <f t="shared" si="2"/>
         <v>-74.120788917090067</v>
       </c>
+      <c r="X20" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.1515859778448478E-2</v>
+      </c>
+      <c r="Y20" s="4"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -2408,12 +2588,21 @@
         <f t="shared" si="0"/>
         <v>-15.530391832549867</v>
       </c>
-      <c r="V21" s="3">
+      <c r="V21" s="4">
         <f t="shared" si="1"/>
+        <v>-6.8514971488908335E-3</v>
+      </c>
+      <c r="W21" s="3">
+        <f t="shared" si="2"/>
         <v>-85.911448442190249</v>
       </c>
+      <c r="X21" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.4816219270780589E-2</v>
+      </c>
+      <c r="Y21" s="4"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -2475,12 +2664,21 @@
         <f t="shared" si="0"/>
         <v>-12.126176146299713</v>
       </c>
-      <c r="V22" s="3">
+      <c r="V22" s="4">
         <f t="shared" si="1"/>
+        <v>-5.4182988271046038E-3</v>
+      </c>
+      <c r="W22" s="3">
+        <f t="shared" si="2"/>
         <v>-62.849656627349759</v>
       </c>
+      <c r="X22" s="4">
+        <f t="shared" si="3"/>
+        <v>-1.8291352149769406E-2</v>
+      </c>
+      <c r="Y22" s="4"/>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -2542,12 +2740,21 @@
         <f t="shared" si="0"/>
         <v>-13.698154733979663</v>
       </c>
-      <c r="V23" s="3">
+      <c r="V23" s="4">
         <f t="shared" si="1"/>
+        <v>-6.0975313446218656E-3</v>
+      </c>
+      <c r="W23" s="3">
+        <f t="shared" si="2"/>
         <v>-77.74240915224982</v>
       </c>
+      <c r="X23" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.2510361990542623E-2</v>
+      </c>
+      <c r="Y23" s="4"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -2609,12 +2816,21 @@
         <f t="shared" si="0"/>
         <v>-11.518024702389994</v>
       </c>
-      <c r="V24" s="3">
+      <c r="V24" s="4">
         <f t="shared" si="1"/>
+        <v>-5.236341020948553E-3</v>
+      </c>
+      <c r="W24" s="3">
+        <f t="shared" si="2"/>
         <v>-74.628131363270313</v>
       </c>
+      <c r="X24" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.23899613404175E-2</v>
+      </c>
+      <c r="Y24" s="4"/>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -2676,12 +2892,21 @@
         <f t="shared" si="0"/>
         <v>-14.82665574793009</v>
       </c>
-      <c r="V25" s="3">
+      <c r="V25" s="4">
         <f t="shared" si="1"/>
+        <v>-6.4965771145187989E-3</v>
+      </c>
+      <c r="W25" s="3">
+        <f t="shared" si="2"/>
         <v>-83.868926477680361</v>
       </c>
+      <c r="X25" s="4">
+        <f t="shared" si="3"/>
+        <v>-2.4383616977775129E-2</v>
+      </c>
+      <c r="Y25" s="4"/>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -2743,12 +2968,21 @@
         <f t="shared" si="0"/>
         <v>-14.856239217520169</v>
       </c>
-      <c r="V26" s="3">
+      <c r="V26" s="4">
         <f t="shared" si="1"/>
+        <v>-9.4216473195375509E-3</v>
+      </c>
+      <c r="W26" s="3">
+        <f t="shared" si="2"/>
         <v>-7.77351280400012</v>
       </c>
+      <c r="X26" s="4">
+        <f t="shared" si="3"/>
+        <v>-4.6607296617251865E-3</v>
+      </c>
+      <c r="Y26" s="4"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -2810,12 +3044,21 @@
         <f t="shared" si="0"/>
         <v>-14.608194468129795</v>
       </c>
-      <c r="V27" s="3">
+      <c r="V27" s="4">
         <f t="shared" si="1"/>
+        <v>-9.2937270134597297E-3</v>
+      </c>
+      <c r="W27" s="3">
+        <f t="shared" si="2"/>
         <v>-7.9449999303801633</v>
       </c>
+      <c r="X27" s="4">
+        <f t="shared" si="3"/>
+        <v>-4.7443199148786966E-3</v>
+      </c>
+      <c r="Y27" s="4"/>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -2877,12 +3120,25 @@
         <f t="shared" si="0"/>
         <v>-14.856239217520169</v>
       </c>
-      <c r="V28" s="3">
+      <c r="V28" s="4">
         <f t="shared" si="1"/>
+        <v>-9.4216473195375509E-3</v>
+      </c>
+      <c r="W28" s="3">
+        <f t="shared" si="2"/>
         <v>-10.198523712230099</v>
       </c>
+      <c r="X28" s="4">
+        <f t="shared" si="3"/>
+        <v>-6.1277639221752854E-3</v>
+      </c>
+      <c r="Y28" s="4"/>
+      <c r="Z28" s="4">
+        <f>AVERAGE(X26:X37)</f>
+        <v>-6.0222811411547658E-3</v>
+      </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>25</v>
       </c>
@@ -2944,12 +3200,21 @@
         <f t="shared" si="0"/>
         <v>-13.68545661538019</v>
       </c>
-      <c r="V29" s="3">
+      <c r="V29" s="4">
         <f t="shared" si="1"/>
+        <v>-8.5985354763262866E-3</v>
+      </c>
+      <c r="W29" s="3">
+        <f t="shared" si="2"/>
         <v>-9.9902478415599489</v>
       </c>
+      <c r="X29" s="4">
+        <f t="shared" si="3"/>
+        <v>-5.9268803133743844E-3</v>
+      </c>
+      <c r="Y29" s="4"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>25</v>
       </c>
@@ -3011,12 +3276,21 @@
         <f t="shared" si="0"/>
         <v>-14.856239217520169</v>
       </c>
-      <c r="V30" s="3">
+      <c r="V30" s="4">
         <f t="shared" si="1"/>
+        <v>-9.4216473195375509E-3</v>
+      </c>
+      <c r="W30" s="3">
+        <f t="shared" si="2"/>
         <v>-12.92415427179003</v>
       </c>
+      <c r="X30" s="4">
+        <f t="shared" si="3"/>
+        <v>-7.7621996496604565E-3</v>
+      </c>
+      <c r="Y30" s="4"/>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>25</v>
       </c>
@@ -3078,12 +3352,21 @@
         <f t="shared" si="0"/>
         <v>-16.221544716139988</v>
       </c>
-      <c r="V31" s="3">
+      <c r="V31" s="4">
         <f t="shared" si="1"/>
+        <v>-9.8693985183095495E-3</v>
+      </c>
+      <c r="W31" s="3">
+        <f t="shared" si="2"/>
         <v>-13.611493728720006</v>
       </c>
+      <c r="X31" s="4">
+        <f t="shared" si="3"/>
+        <v>-7.8481276765771917E-3</v>
+      </c>
+      <c r="Y31" s="4"/>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>25</v>
       </c>
@@ -3145,12 +3428,21 @@
         <f t="shared" si="0"/>
         <v>-14.856239217520169</v>
       </c>
-      <c r="V32" s="3">
+      <c r="V32" s="4">
         <f t="shared" si="1"/>
+        <v>-9.4216473195375509E-3</v>
+      </c>
+      <c r="W32" s="3">
+        <f t="shared" si="2"/>
         <v>-7.4985141252000176</v>
       </c>
+      <c r="X32" s="4">
+        <f t="shared" si="3"/>
+        <v>-4.4846035950570498E-3</v>
+      </c>
+      <c r="Y32" s="4"/>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>25</v>
       </c>
@@ -3212,12 +3504,21 @@
         <f t="shared" si="0"/>
         <v>-15.949227363079899</v>
       </c>
-      <c r="V33" s="3">
+      <c r="V33" s="4">
         <f t="shared" si="1"/>
+        <v>-1.0023232939282143E-2</v>
+      </c>
+      <c r="W33" s="3">
+        <f t="shared" si="2"/>
         <v>-10.500546976709984</v>
       </c>
+      <c r="X33" s="4">
+        <f t="shared" si="3"/>
+        <v>-6.223617781310105E-3</v>
+      </c>
+      <c r="Y33" s="4"/>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>25</v>
       </c>
@@ -3279,12 +3580,21 @@
         <f t="shared" si="0"/>
         <v>-14.856239217520169</v>
       </c>
-      <c r="V34" s="3">
+      <c r="V34" s="4">
         <f t="shared" si="1"/>
+        <v>-9.4216473195375509E-3</v>
+      </c>
+      <c r="W34" s="3">
+        <f t="shared" si="2"/>
         <v>-8.9664732982701025</v>
       </c>
+      <c r="X34" s="4">
+        <f t="shared" si="3"/>
+        <v>-5.3762029711775204E-3</v>
+      </c>
+      <c r="Y34" s="4"/>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>25</v>
       </c>
@@ -3346,12 +3656,21 @@
         <f t="shared" si="0"/>
         <v>-15.546452207560151</v>
       </c>
-      <c r="V35" s="3">
+      <c r="V35" s="4">
         <f t="shared" si="1"/>
+        <v>-9.8379526021270744E-3</v>
+      </c>
+      <c r="W35" s="3">
+        <f t="shared" si="2"/>
         <v>-13.332955914670038</v>
       </c>
+      <c r="X35" s="4">
+        <f t="shared" si="3"/>
+        <v>-7.9666492642273927E-3</v>
+      </c>
+      <c r="Y35" s="4"/>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -3413,12 +3732,21 @@
         <f t="shared" si="0"/>
         <v>-14.856239217520169</v>
       </c>
-      <c r="V36" s="3">
+      <c r="V36" s="4">
         <f t="shared" si="1"/>
+        <v>-9.4216473195375509E-3</v>
+      </c>
+      <c r="W36" s="3">
+        <f t="shared" si="2"/>
         <v>-9.4717060459299773</v>
       </c>
+      <c r="X36" s="4">
+        <f t="shared" si="3"/>
+        <v>-5.7384233635478996E-3</v>
+      </c>
+      <c r="Y36" s="4"/>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>25</v>
       </c>
@@ -3480,10 +3808,19 @@
         <f t="shared" si="0"/>
         <v>-15.103435203019899</v>
       </c>
-      <c r="V37" s="3">
+      <c r="V37" s="4">
         <f t="shared" si="1"/>
+        <v>-9.3023955167303007E-3</v>
+      </c>
+      <c r="W37" s="3">
+        <f t="shared" si="2"/>
         <v>-9.2340565298400179</v>
       </c>
+      <c r="X37" s="4">
+        <f t="shared" si="3"/>
+        <v>-5.4078555801459986E-3</v>
+      </c>
+      <c r="Y37" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>